<commit_message>
[IMP] template xlsx export bom
</commit_message>
<xml_diff>
--- a/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
+++ b/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">Product</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t xml:space="preserve">Bom Lines / Unit of Measure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(bom_line/product_name)</t>
   </si>
 </sst>
 </file>
@@ -219,15 +222,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ1"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24.73"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -251,6 +255,9 @@
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="ALW1" s="0"/>
       <c r="ALX1" s="0"/>

</xml_diff>

<commit_message>
[IMP] remove u.m. from export/import logic
</commit_message>
<xml_diff>
--- a/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
+++ b/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="mrp_bom" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="mrp_bom" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">Product</t>
   </si>
@@ -28,9 +28,6 @@
     <t xml:space="preserve">Quantity</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit of Measure</t>
-  </si>
-  <si>
     <t xml:space="preserve">Routing</t>
   </si>
   <si>
@@ -38,9 +35,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bom Lines / Quantity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Unit of Measure</t>
   </si>
   <si>
     <t xml:space="preserve">(bom_line/product_name)</t>
@@ -131,16 +125,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -216,61 +214,161 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ1"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.73"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="ALW1" s="0"/>
-      <c r="ALX1" s="0"/>
-      <c r="ALY1" s="0"/>
-      <c r="ALZ1" s="0"/>
-      <c r="AMA1" s="0"/>
-      <c r="AMB1" s="0"/>
-      <c r="AMC1" s="0"/>
-      <c r="AMD1" s="0"/>
-      <c r="AME1" s="0"/>
-      <c r="AMF1" s="0"/>
-      <c r="AMG1" s="0"/>
-      <c r="AMH1" s="0"/>
+      <c r="ALU1" s="1"/>
+      <c r="ALV1" s="1"/>
+      <c r="ALW1" s="1"/>
+      <c r="ALX1" s="1"/>
+      <c r="ALY1" s="1"/>
+      <c r="ALZ1" s="1"/>
+      <c r="AMA1" s="1"/>
+      <c r="AMB1" s="1"/>
+      <c r="AMC1" s="1"/>
+      <c r="AMD1" s="1"/>
+      <c r="AME1" s="1"/>
+      <c r="AMF1" s="1"/>
+      <c r="AMG1" s="1"/>
+      <c r="AMH1" s="1"/>
       <c r="AMI1" s="0"/>
       <c r="AMJ1" s="0"/>
     </row>

</xml_diff>

<commit_message>
[IMP] add other columns to excel_import_export_bom
</commit_message>
<xml_diff>
--- a/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
+++ b/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">Product</t>
   </si>
@@ -37,7 +37,49 @@
     <t xml:space="preserve">Bom Lines / Quantity</t>
   </si>
   <si>
-    <t xml:space="preserve">(bom_line/product_name)</t>
+    <t xml:space="preserve">Bom Lines / Product Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Manufacturer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Manufacturer Product Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Manufacturer Product Reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Manufacturer Product URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Model (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Power (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Voltage (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Output (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Range (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / T. Work (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Electric Connection (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Hydraulic Connection (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / Material (electric info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bom Lines / P&amp;ID (electric info)</t>
   </si>
 </sst>
 </file>
@@ -333,7 +375,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.11"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -352,8 +394,50 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="ALU1" s="1"/>
       <c r="ALV1" s="1"/>
@@ -369,8 +453,8 @@
       <c r="AMF1" s="1"/>
       <c r="AMG1" s="1"/>
       <c r="AMH1" s="1"/>
-      <c r="AMI1" s="0"/>
-      <c r="AMJ1" s="0"/>
+      <c r="AMI1" s="1"/>
+      <c r="AMJ1" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Revert "[IMP] add other columns to excel_import_export_bom"
This reverts commit e9a2ae4a2fa41f58fb9be66038697799eb92e9b3.
</commit_message>
<xml_diff>
--- a/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
+++ b/excel_import_export_bom/import_export_mrp_bom/mrp_bom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">Product</t>
   </si>
@@ -37,49 +37,7 @@
     <t xml:space="preserve">Bom Lines / Quantity</t>
   </si>
   <si>
-    <t xml:space="preserve">Bom Lines / Product Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Manufacturer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Manufacturer Product Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Manufacturer Product Reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Manufacturer Product URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Model (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Power (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Voltage (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Output (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Range (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / T. Work (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Electric Connection (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Hydraulic Connection (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / Material (electric info)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bom Lines / P&amp;ID (electric info)</t>
+    <t xml:space="preserve">(bom_line/product_name)</t>
   </si>
 </sst>
 </file>
@@ -375,7 +333,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.73"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -394,50 +352,8 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="ALU1" s="1"/>
       <c r="ALV1" s="1"/>
@@ -453,8 +369,8 @@
       <c r="AMF1" s="1"/>
       <c r="AMG1" s="1"/>
       <c r="AMH1" s="1"/>
-      <c r="AMI1" s="1"/>
-      <c r="AMJ1" s="1"/>
+      <c r="AMI1" s="0"/>
+      <c r="AMJ1" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>